<commit_message>
final report output refinement
</commit_message>
<xml_diff>
--- a/data/processed/sam_auto_dashboard_2024_refresh/occ_change_by_education/total_occ_change_by_education_2021_2024_auto.xlsx
+++ b/data/processed/sam_auto_dashboard_2024_refresh/occ_change_by_education/total_occ_change_by_education_2021_2024_auto.xlsx
@@ -1,17 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vasilauskas\GitHub\EV-Transition\data\processed\sam_auto_dashboard_2024_refresh\occ_change_by_education\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01098B0C-117B-4F63-9FE3-6D84A85516CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Education" sheetId="1" r:id="rId1"/>
     <sheet name="Education+Training" sheetId="2" r:id="rId2"/>
     <sheet name="Edu+Training (custom)" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -96,8 +115,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +126,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -146,27 +172,38 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -204,7 +241,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -238,6 +275,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -272,9 +310,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -447,11 +486,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,7 +525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -500,7 +539,7 @@
         <v>14</v>
       </c>
       <c r="E2">
-        <v>59515.86626028</v>
+        <v>59515.866260280003</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
@@ -512,7 +551,7 @@
         <v>19</v>
       </c>
       <c r="I2">
-        <v>70121.14510613833</v>
+        <v>70121.145106138327</v>
       </c>
       <c r="J2">
         <v>10605.27884585832</v>
@@ -521,7 +560,7 @@
         <v>0.1781924638293659</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -535,7 +574,7 @@
         <v>15</v>
       </c>
       <c r="E3">
-        <v>324357.2425995042</v>
+        <v>324357.24259950418</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
@@ -547,16 +586,16 @@
         <v>19</v>
       </c>
       <c r="I3">
-        <v>328638.4390227165</v>
+        <v>328638.43902271648</v>
       </c>
       <c r="J3">
-        <v>4281.196423212299</v>
+        <v>4281.1964232122991</v>
       </c>
       <c r="K3">
-        <v>0.01319901596431577</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>1.3199015964315769E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -570,7 +609,7 @@
         <v>16</v>
       </c>
       <c r="E4">
-        <v>66466.93868361582</v>
+        <v>66466.938683615823</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -582,13 +621,13 @@
         <v>19</v>
       </c>
       <c r="I4">
-        <v>64622.30597480127</v>
+        <v>64622.305974801267</v>
       </c>
       <c r="J4">
-        <v>-1844.632708814548</v>
+        <v>-1844.6327088145481</v>
       </c>
       <c r="K4">
-        <v>-0.02775263530031137</v>
+        <v>-2.7752635300311371E-2</v>
       </c>
     </row>
   </sheetData>
@@ -597,11 +636,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -636,7 +675,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -650,7 +689,7 @@
         <v>14</v>
       </c>
       <c r="E2">
-        <v>59515.86626028</v>
+        <v>59515.866260280003</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
@@ -662,7 +701,7 @@
         <v>19</v>
       </c>
       <c r="I2">
-        <v>70121.14510613833</v>
+        <v>70121.145106138327</v>
       </c>
       <c r="J2">
         <v>10605.27884585832</v>
@@ -671,7 +710,7 @@
         <v>0.1781924638293659</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -697,16 +736,16 @@
         <v>19</v>
       </c>
       <c r="I3">
-        <v>135483.1360098894</v>
+        <v>135483.13600988939</v>
       </c>
       <c r="J3">
-        <v>7071.235970345137</v>
+        <v>7071.2359703451366</v>
       </c>
       <c r="K3">
-        <v>0.05506682767070312</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>5.5066827670703117E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -720,7 +759,7 @@
         <v>21</v>
       </c>
       <c r="E4">
-        <v>262412.2812435757</v>
+        <v>262412.28124357568</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -732,13 +771,13 @@
         <v>19</v>
       </c>
       <c r="I4">
-        <v>257777.6089876284</v>
+        <v>257777.60898762839</v>
       </c>
       <c r="J4">
         <v>-4634.672255947371</v>
       </c>
       <c r="K4">
-        <v>-0.01766179629239756</v>
+        <v>-1.7661796292397561E-2</v>
       </c>
     </row>
   </sheetData>
@@ -747,11 +786,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -786,7 +825,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -800,7 +839,7 @@
         <v>22</v>
       </c>
       <c r="E2">
-        <v>3777.178100521485</v>
+        <v>3777.1781005214848</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
@@ -812,16 +851,16 @@
         <v>19</v>
       </c>
       <c r="I2">
-        <v>4865.075944256964</v>
+        <v>4865.0759442569642</v>
       </c>
       <c r="J2">
         <v>1087.897843735479</v>
       </c>
-      <c r="K2">
-        <v>0.2880186781728089</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="K2" s="2">
+        <v>0.28801867817280891</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -835,7 +874,7 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>59515.86626028</v>
+        <v>59515.866260280003</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
@@ -847,16 +886,16 @@
         <v>19</v>
       </c>
       <c r="I3">
-        <v>70121.14510613833</v>
+        <v>70121.145106138327</v>
       </c>
       <c r="J3">
         <v>10605.27884585832</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="2">
         <v>0.1781924638293659</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -870,7 +909,7 @@
         <v>23</v>
       </c>
       <c r="E4">
-        <v>206788.0996220559</v>
+        <v>206788.09962205589</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -882,16 +921,16 @@
         <v>19</v>
       </c>
       <c r="I4">
-        <v>204301.4423440537</v>
+        <v>204301.44234405371</v>
       </c>
       <c r="J4">
-        <v>-2486.657278002269</v>
-      </c>
-      <c r="K4">
-        <v>-0.01202514691390414</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>-2486.6572780022689</v>
+      </c>
+      <c r="K4" s="2">
+        <v>-1.202514691390414E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -905,7 +944,7 @@
         <v>24</v>
       </c>
       <c r="E5">
-        <v>180258.9035605426</v>
+        <v>180258.90356054259</v>
       </c>
       <c r="F5" t="s">
         <v>17</v>
@@ -917,13 +956,13 @@
         <v>19</v>
       </c>
       <c r="I5">
-        <v>184094.2267092071</v>
+        <v>184094.22670920711</v>
       </c>
       <c r="J5">
-        <v>3835.323148664524</v>
-      </c>
-      <c r="K5">
-        <v>0.02127674735010454</v>
+        <v>3835.3231486645241</v>
+      </c>
+      <c r="K5" s="2">
+        <v>2.1276747350104541E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>